<commit_message>
feat: add way to transcribe file instead of recording
</commit_message>
<xml_diff>
--- a/data/translation_times.xlsx
+++ b/data/translation_times.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\repos\translator-helper\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F9F29EC-D8BD-42D8-B1AE-8978707B9DE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35C6D481-5497-4B5C-9C43-1F29DB8264B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{50C1EBFE-BD10-47AD-808E-F15717A1EC41}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="31">
   <si>
     <t>video</t>
   </si>
@@ -57,9 +57,6 @@
     <t>average_character_count</t>
   </si>
   <si>
-    <t>context_size</t>
-  </si>
-  <si>
     <t>cost_usd</t>
   </si>
   <si>
@@ -117,10 +114,19 @@
     <t>gakumas lilja white night white wish</t>
   </si>
   <si>
-    <t>gakumas</t>
-  </si>
-  <si>
     <t>gpt-4.1-mini</t>
+  </si>
+  <si>
+    <t>gakumas event 01</t>
+  </si>
+  <si>
+    <t>batch_size</t>
+  </si>
+  <si>
+    <t>gakumas lilja step 3</t>
+  </si>
+  <si>
+    <t>claude sonnet 4.6</t>
   </si>
 </sst>
 </file>
@@ -498,7 +504,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B2B118A-139E-42B7-BCC2-032941E226DF}">
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:O15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="8.28515625" customWidth="1"/>
@@ -511,7 +517,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
@@ -532,24 +538,24 @@
         <v>6</v>
       </c>
       <c r="I1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" t="s">
-        <v>9</v>
-      </c>
       <c r="L1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -586,19 +592,19 @@
         <v>2.5668449197860967E-3</v>
       </c>
       <c r="N2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="O2">
         <f>AVERAGE(L:L)</f>
-        <v>2.5487497783481801E-3</v>
+        <v>2.418331334627957E-3</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -628,19 +634,19 @@
         <v>2.1985815602836882E-3</v>
       </c>
       <c r="N3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="O3">
         <f>SUM(F:F)</f>
-        <v>4636</v>
+        <v>5051</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -678,10 +684,10 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -719,10 +725,10 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -760,10 +766,10 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -801,10 +807,10 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -842,10 +848,10 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C9">
         <v>0</v>
@@ -883,10 +889,10 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -924,10 +930,10 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -965,10 +971,10 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C12">
         <v>0</v>
@@ -1006,10 +1012,10 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B13" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C13">
         <v>0</v>
@@ -1047,10 +1053,10 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B14" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -1079,12 +1085,53 @@
         <v>1.24</v>
       </c>
       <c r="K14" s="2">
-        <f t="shared" ref="K14" si="3">J14/G14</f>
+        <f t="shared" ref="K14:K15" si="3">J14/G14</f>
         <v>7.7311553089344715E-5</v>
       </c>
       <c r="L14">
-        <f t="shared" ref="L14" si="4">J14/F14</f>
+        <f t="shared" ref="L14:L15" si="4">J14/F14</f>
         <v>1.7971014492753623E-3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>3</v>
+      </c>
+      <c r="E15">
+        <v>17</v>
+      </c>
+      <c r="F15" s="3">
+        <v>415</v>
+      </c>
+      <c r="G15" s="3">
+        <v>8506</v>
+      </c>
+      <c r="H15" s="1">
+        <f>G15/F15</f>
+        <v>20.496385542168674</v>
+      </c>
+      <c r="I15">
+        <v>50</v>
+      </c>
+      <c r="J15">
+        <v>0.3</v>
+      </c>
+      <c r="K15" s="2">
+        <f t="shared" si="3"/>
+        <v>3.526922172584058E-5</v>
+      </c>
+      <c r="L15">
+        <f t="shared" si="4"/>
+        <v>7.2289156626506026E-4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: move task logic to their own files
</commit_message>
<xml_diff>
--- a/data/translation_times.xlsx
+++ b/data/translation_times.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\repos\translator-helper\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35C6D481-5497-4B5C-9C43-1F29DB8264B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD6333A4-7494-42FF-B237-D06DDBA161AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{50C1EBFE-BD10-47AD-808E-F15717A1EC41}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{50C1EBFE-BD10-47AD-808E-F15717A1EC41}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="33">
   <si>
     <t>video</t>
   </si>
@@ -127,6 +127,12 @@
   </si>
   <si>
     <t>claude sonnet 4.6</t>
+  </si>
+  <si>
+    <t>gakumas event 02</t>
+  </si>
+  <si>
+    <t>gakumas tokimeki emotion lilja</t>
   </si>
 </sst>
 </file>
@@ -504,7 +510,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B2B118A-139E-42B7-BCC2-032941E226DF}">
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:O17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="8.28515625" customWidth="1"/>
@@ -596,7 +602,7 @@
       </c>
       <c r="O2">
         <f>AVERAGE(L:L)</f>
-        <v>2.418331334627957E-3</v>
+        <v>2.2092027773925084E-3</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -638,7 +644,7 @@
       </c>
       <c r="O3">
         <f>SUM(F:F)</f>
-        <v>5051</v>
+        <v>5761</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -1085,11 +1091,11 @@
         <v>1.24</v>
       </c>
       <c r="K14" s="2">
-        <f t="shared" ref="K14:K15" si="3">J14/G14</f>
+        <f t="shared" ref="K14:K17" si="3">J14/G14</f>
         <v>7.7311553089344715E-5</v>
       </c>
       <c r="L14">
-        <f t="shared" ref="L14:L15" si="4">J14/F14</f>
+        <f t="shared" ref="L14:L17" si="4">J14/F14</f>
         <v>1.7971014492753623E-3</v>
       </c>
     </row>
@@ -1132,6 +1138,89 @@
       <c r="L15">
         <f t="shared" si="4"/>
         <v>7.2289156626506026E-4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16">
+        <v>0</v>
+      </c>
+      <c r="D16">
+        <v>4</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="F16" s="3">
+        <v>508</v>
+      </c>
+      <c r="G16" s="3">
+        <v>10965</v>
+      </c>
+      <c r="H16" s="1">
+        <f>G16/F16</f>
+        <v>21.584645669291337</v>
+      </c>
+      <c r="I16">
+        <v>50</v>
+      </c>
+      <c r="J16">
+        <v>0.38</v>
+      </c>
+      <c r="K16" s="2">
+        <f t="shared" si="3"/>
+        <v>3.4655722754217965E-5</v>
+      </c>
+      <c r="L16">
+        <f t="shared" si="4"/>
+        <v>7.4803149606299214E-4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17">
+        <v>0</v>
+      </c>
+      <c r="D17">
+        <v>1</v>
+      </c>
+      <c r="E17">
+        <v>33</v>
+      </c>
+      <c r="F17" s="3">
+        <v>202</v>
+      </c>
+      <c r="G17" s="3">
+        <v>4725</v>
+      </c>
+      <c r="H17" s="1">
+        <f>G17/F17</f>
+        <v>23.39108910891089</v>
+      </c>
+      <c r="I17">
+        <v>50</v>
+      </c>
+      <c r="J17">
+        <f>0.22-0.07</f>
+        <v>0.15</v>
+      </c>
+      <c r="K17" s="2">
+        <f t="shared" si="3"/>
+        <v>3.1746031746031745E-5</v>
+      </c>
+      <c r="L17">
+        <f t="shared" si="4"/>
+        <v>7.4257425742574258E-4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: update file translation task and show errors in frontend
</commit_message>
<xml_diff>
--- a/data/translation_times.xlsx
+++ b/data/translation_times.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\repos\translator-helper\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD6333A4-7494-42FF-B237-D06DDBA161AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B8620B4-C926-4BC5-B35D-A33D514F80A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{50C1EBFE-BD10-47AD-808E-F15717A1EC41}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{50C1EBFE-BD10-47AD-808E-F15717A1EC41}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="35">
   <si>
     <t>video</t>
   </si>
@@ -133,6 +133,12 @@
   </si>
   <si>
     <t>gakumas tokimeki emotion lilja</t>
+  </si>
+  <si>
+    <t>gakumas event 03</t>
+  </si>
+  <si>
+    <t>claude haiku 4.5</t>
   </si>
 </sst>
 </file>
@@ -142,10 +148,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -510,7 +522,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B2B118A-139E-42B7-BCC2-032941E226DF}">
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:O21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="8.28515625" customWidth="1"/>
@@ -602,7 +614,7 @@
       </c>
       <c r="O2">
         <f>AVERAGE(L:L)</f>
-        <v>2.2092027773925084E-3</v>
+        <v>1.831961705118141E-3</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -644,7 +656,7 @@
       </c>
       <c r="O3">
         <f>SUM(F:F)</f>
-        <v>5761</v>
+        <v>7309</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -998,7 +1010,7 @@
         <v>2620</v>
       </c>
       <c r="H12" s="1">
-        <f>G12/F12</f>
+        <f t="shared" ref="H12:H19" si="3">G12/F12</f>
         <v>16.073619631901842</v>
       </c>
       <c r="I12">
@@ -1039,7 +1051,7 @@
         <v>5706</v>
       </c>
       <c r="H13" s="1">
-        <f>G13/F13</f>
+        <f t="shared" si="3"/>
         <v>23.578512396694215</v>
       </c>
       <c r="I13">
@@ -1080,7 +1092,7 @@
         <v>16039</v>
       </c>
       <c r="H14" s="1">
-        <f>G14/F14</f>
+        <f t="shared" si="3"/>
         <v>23.244927536231884</v>
       </c>
       <c r="I14">
@@ -1091,11 +1103,11 @@
         <v>1.24</v>
       </c>
       <c r="K14" s="2">
-        <f t="shared" ref="K14:K17" si="3">J14/G14</f>
+        <f t="shared" ref="K14:K18" si="4">J14/G14</f>
         <v>7.7311553089344715E-5</v>
       </c>
       <c r="L14">
-        <f t="shared" ref="L14:L17" si="4">J14/F14</f>
+        <f t="shared" ref="L14:L18" si="5">J14/F14</f>
         <v>1.7971014492753623E-3</v>
       </c>
     </row>
@@ -1122,7 +1134,7 @@
         <v>8506</v>
       </c>
       <c r="H15" s="1">
-        <f>G15/F15</f>
+        <f t="shared" si="3"/>
         <v>20.496385542168674</v>
       </c>
       <c r="I15">
@@ -1132,11 +1144,11 @@
         <v>0.3</v>
       </c>
       <c r="K15" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>3.526922172584058E-5</v>
       </c>
       <c r="L15">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>7.2289156626506026E-4</v>
       </c>
     </row>
@@ -1163,7 +1175,7 @@
         <v>10965</v>
       </c>
       <c r="H16" s="1">
-        <f>G16/F16</f>
+        <f t="shared" si="3"/>
         <v>21.584645669291337</v>
       </c>
       <c r="I16">
@@ -1173,11 +1185,11 @@
         <v>0.38</v>
       </c>
       <c r="K16" s="2">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>3.4655722754217965E-5</v>
       </c>
       <c r="L16">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>7.4803149606299214E-4</v>
       </c>
     </row>
@@ -1204,7 +1216,7 @@
         <v>4725</v>
       </c>
       <c r="H17" s="1">
-        <f>G17/F17</f>
+        <f t="shared" si="3"/>
         <v>23.39108910891089</v>
       </c>
       <c r="I17">
@@ -1215,15 +1227,184 @@
         <v>0.15</v>
       </c>
       <c r="K17" s="2">
+        <f t="shared" si="4"/>
+        <v>3.1746031746031745E-5</v>
+      </c>
+      <c r="L17">
+        <f t="shared" si="5"/>
+        <v>7.4257425742574258E-4</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>33</v>
+      </c>
+      <c r="B18" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18">
+        <v>0</v>
+      </c>
+      <c r="D18">
+        <v>2</v>
+      </c>
+      <c r="E18">
+        <v>6</v>
+      </c>
+      <c r="F18" s="3">
+        <v>387</v>
+      </c>
+      <c r="G18" s="3">
+        <v>8158</v>
+      </c>
+      <c r="H18" s="1">
         <f t="shared" si="3"/>
-        <v>3.1746031746031745E-5</v>
-      </c>
-      <c r="L17">
+        <v>21.080103359173126</v>
+      </c>
+      <c r="I18">
+        <v>50</v>
+      </c>
+      <c r="J18">
+        <f>0.83-0.71</f>
+        <v>0.12</v>
+      </c>
+      <c r="K18" s="2">
         <f t="shared" si="4"/>
-        <v>7.4257425742574258E-4</v>
+        <v>1.4709487619514587E-5</v>
+      </c>
+      <c r="L18">
+        <f t="shared" si="5"/>
+        <v>3.1007751937984492E-4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" t="s">
+        <v>34</v>
+      </c>
+      <c r="C19">
+        <v>0</v>
+      </c>
+      <c r="D19">
+        <v>2</v>
+      </c>
+      <c r="E19">
+        <v>4</v>
+      </c>
+      <c r="F19" s="3">
+        <v>387</v>
+      </c>
+      <c r="G19" s="3">
+        <v>8158</v>
+      </c>
+      <c r="H19" s="1">
+        <f t="shared" si="3"/>
+        <v>21.080103359173126</v>
+      </c>
+      <c r="I19">
+        <v>50</v>
+      </c>
+      <c r="J19">
+        <f>0.71-0.57</f>
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="K19" s="2">
+        <f t="shared" ref="K19" si="6">J19/G19</f>
+        <v>1.7161068889433685E-5</v>
+      </c>
+      <c r="L19">
+        <f t="shared" ref="L19" si="7">J19/F19</f>
+        <v>3.6175710594315251E-4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>33</v>
+      </c>
+      <c r="B20" t="s">
+        <v>34</v>
+      </c>
+      <c r="C20">
+        <v>0</v>
+      </c>
+      <c r="D20">
+        <v>2</v>
+      </c>
+      <c r="E20">
+        <v>6</v>
+      </c>
+      <c r="F20" s="3">
+        <v>387</v>
+      </c>
+      <c r="G20" s="3">
+        <v>8158</v>
+      </c>
+      <c r="H20" s="1">
+        <f t="shared" ref="H20:H21" si="8">G20/F20</f>
+        <v>21.080103359173126</v>
+      </c>
+      <c r="I20">
+        <v>50</v>
+      </c>
+      <c r="J20">
+        <f>0.95-0.83</f>
+        <v>0.12</v>
+      </c>
+      <c r="K20" s="2">
+        <f t="shared" ref="K20" si="9">J20/G20</f>
+        <v>1.4709487619514587E-5</v>
+      </c>
+      <c r="L20">
+        <f t="shared" ref="L20" si="10">J20/F20</f>
+        <v>3.1007751937984492E-4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>33</v>
+      </c>
+      <c r="B21" t="s">
+        <v>34</v>
+      </c>
+      <c r="C21">
+        <v>0</v>
+      </c>
+      <c r="D21">
+        <v>2</v>
+      </c>
+      <c r="E21">
+        <v>6</v>
+      </c>
+      <c r="F21" s="3">
+        <v>387</v>
+      </c>
+      <c r="G21" s="3">
+        <v>8158</v>
+      </c>
+      <c r="H21" s="1">
+        <f t="shared" si="8"/>
+        <v>21.080103359173126</v>
+      </c>
+      <c r="I21">
+        <v>50</v>
+      </c>
+      <c r="J21">
+        <f>1.07-0.95</f>
+        <v>0.12000000000000011</v>
+      </c>
+      <c r="K21" s="2">
+        <f t="shared" ref="K21" si="11">J21/G21</f>
+        <v>1.47094876195146E-5</v>
+      </c>
+      <c r="L21">
+        <f t="shared" ref="L21" si="12">J21/F21</f>
+        <v>3.1007751937984525E-4</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add review translated file feature
</commit_message>
<xml_diff>
--- a/data/translation_times.xlsx
+++ b/data/translation_times.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\repos\translator-helper\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B8620B4-C926-4BC5-B35D-A33D514F80A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B58608F0-7AA9-4880-B359-2725A5B2571B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{50C1EBFE-BD10-47AD-808E-F15717A1EC41}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{50C1EBFE-BD10-47AD-808E-F15717A1EC41}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="36">
   <si>
     <t>video</t>
   </si>
@@ -139,6 +139,9 @@
   </si>
   <si>
     <t>claude haiku 4.5</t>
+  </si>
+  <si>
+    <t>gakumas event 04</t>
   </si>
 </sst>
 </file>
@@ -522,7 +525,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B2B118A-139E-42B7-BCC2-032941E226DF}">
-  <dimension ref="A1:O21"/>
+  <dimension ref="A1:O22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="8.28515625" customWidth="1"/>
@@ -614,7 +617,7 @@
       </c>
       <c r="O2">
         <f>AVERAGE(L:L)</f>
-        <v>1.831961705118141E-3</v>
+        <v>1.755255443975859E-3</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -656,7 +659,7 @@
       </c>
       <c r="O3">
         <f>SUM(F:F)</f>
-        <v>7309</v>
+        <v>7716</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
@@ -1342,7 +1345,7 @@
         <v>8158</v>
       </c>
       <c r="H20" s="1">
-        <f t="shared" ref="H20:H21" si="8">G20/F20</f>
+        <f t="shared" ref="H20:H22" si="8">G20/F20</f>
         <v>21.080103359173126</v>
       </c>
       <c r="I20">
@@ -1395,12 +1398,53 @@
         <v>0.12000000000000011</v>
       </c>
       <c r="K21" s="2">
-        <f t="shared" ref="K21" si="11">J21/G21</f>
+        <f>J21/G21</f>
         <v>1.47094876195146E-5</v>
       </c>
       <c r="L21">
-        <f t="shared" ref="L21" si="12">J21/F21</f>
+        <f t="shared" ref="L21" si="11">J21/F21</f>
         <v>3.1007751937984525E-4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>35</v>
+      </c>
+      <c r="B22" t="s">
+        <v>34</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+      <c r="D22">
+        <v>1</v>
+      </c>
+      <c r="E22">
+        <v>39</v>
+      </c>
+      <c r="F22" s="3">
+        <v>407</v>
+      </c>
+      <c r="G22" s="3">
+        <v>8318</v>
+      </c>
+      <c r="H22" s="1">
+        <f t="shared" si="8"/>
+        <v>20.437346437346438</v>
+      </c>
+      <c r="I22">
+        <v>50</v>
+      </c>
+      <c r="J22">
+        <v>0.09</v>
+      </c>
+      <c r="K22" s="2">
+        <f>J22/G22</f>
+        <v>1.0819908631882663E-5</v>
+      </c>
+      <c r="L22">
+        <f t="shared" ref="L22" si="12">J22/F22</f>
+        <v>2.2113022113022111E-4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>